<commit_message>
fixed pinout and added fuse detection
</commit_message>
<xml_diff>
--- a/docs/SPS SMS Commands.xlsx
+++ b/docs/SPS SMS Commands.xlsx
@@ -26,6 +26,7 @@
     <sheet name="SPA Roadmap" sheetId="7" r:id="rId11"/>
     <sheet name="JSON Format" sheetId="10" r:id="rId12"/>
     <sheet name="SPA Display" sheetId="11" r:id="rId13"/>
+    <sheet name="Fuse Detection Alert" sheetId="16" r:id="rId18"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -31055,6 +31056,220 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:B16"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="28" customWidth="1"/>
+    <col min="2" max="2" width="110" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SPS Fuse Detection Alert</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Behavior</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Input GPIO</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P1.12 / BL54L15 module pad 34; active-low GPIO input.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LED GPIOs</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Utility LED P2.08; cellular LED P2.09.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Circuit</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LTV-814; external 47 kohm pull-up to 3.3 V; 100 nF RC filter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sampling</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Look for an active-low pulse over up to 40 ms, sampling about every 1 ms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wiring assumption</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AC_IN before the fuse; socket metering after the fuse.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Trigger</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Input AC present and all socket metering channels below 50 V for three consecutive network-ready alert polls.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alert payload</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alert=Utility power lost - fuse probably blown
+Utility=OFF
+Device=0110
+Outlet=1111
+RSL=-101
+Batt=4.44
+Lat=42.027998
+Lon=-91.631620
+FW=001.00
+HBD=0.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No upstream AC</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Existing Utility power lost alert; no fuse diagnosis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Input AC returns alone</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirm and send probable fuse alert even during an existing utility outage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Retry and duplicates</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Retry failed sends; send successful fuse alert once until socket voltage returns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Restoration</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Existing Utility power restored alert and outlet report.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No outlet report</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The loss/fuse alert is not followed by an outlet report.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No new incoming command</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This is an automatic alert.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Diagnosis limitation</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Metering faults or another downstream interruption can produce the same symptoms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Full documentation</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">docs/all_cmds.md and docs/sms_commands_client.html</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{707EC4CB-5D5A-4E5D-B024-2AA3920762A0}">
   <dimension ref="A1:F63"/>

</xml_diff>

<commit_message>
took more robust approach
</commit_message>
<xml_diff>
--- a/docs/SPS SMS Commands.xlsx
+++ b/docs/SPS SMS Commands.xlsx
@@ -31309,7 +31309,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -31549,6 +31549,42 @@
       <c r="B19" t="inlineStr">
         <is>
           <t xml:space="preserve">Boot logs MX25R6435FZNIL0, JEDEC c2 28 17 and 8 MiB capacity. Each save is read back and compared; logs persisted and verified or an error.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Relay command errors</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>DeviceOn/DeviceOff return ERR ... GPIO or ERR ... save when switching/persistence fails; outputs may already have changed. Reboot commands report save failures.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Repeated relay commands</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Already-correct outputs skip GPIO writes. A mask matching the last loaded/verified saved mask skips flash access; failed saves invalidate that cache.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Relay reset diagnostics</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Boot reset-cause flags plus relay, settings write/readback and SMS-reply stage logs. See Relay_restart_diagnostics.md. Root cause of reported restarts is not yet confirmed.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fixed signing key issue
</commit_message>
<xml_diff>
--- a/docs/SPS SMS Commands.xlsx
+++ b/docs/SPS SMS Commands.xlsx
@@ -31828,7 +31828,7 @@
 Run=Internal
 From=Backup B
 Backup=Ready
-Health=OK/60s
+Health=Off
 Boots=12 WDT=3
 Streak=0/3
 Recoveries=1
@@ -31857,7 +31857,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ready means header/length/CRC and signature against either project public key pass a fresh readback. None=not provisioned, Bad=verification failed. The first healthy run reprovisions an intact B signed outside the new trust set after the SWD transition.</t>
+          <t xml:space="preserve">Ready means header/length/CRC and signature against either project public key pass a fresh readback. None=not provisioned, Bad=verification failed. Startup backup provisioning is disabled. Update preparation authenticates and archives the running image to B before erasing A, replacing an old SDK-signed backup then.</t>
         </is>
       </c>
     </row>
@@ -31869,7 +31869,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wait/60s or OK/60s; one minute for testing after completed main-loop progress with settings and verified backup. Production can use 300000U.</t>
+          <t xml:space="preserve">Off: startup health check disabled (CONFIG_SPS_OTA_HEALTH_CHECK=n). OTA has no 60-second health prerequisite. Backup creation and signature checks remain mandatory during update preparation.</t>
         </is>
       </c>
     </row>
@@ -31893,7 +31893,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Current consecutive watchdog failure count / 3. Cleared by healthy check or non-watchdog restart.</t>
+          <t xml:space="preserve">Current consecutive watchdog failure count / 3. Cleared after one minute of sustained main-loop progress or a non-watchdog restart, independently of the disabled OTA health check.</t>
         </is>
       </c>
     </row>
@@ -31905,7 +31905,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Completed restorations and latest completed reason: Watchdog, Image (boot/validation failure), None. History survives healthy check and normal reboot.</t>
+          <t xml:space="preserve">Completed restorations and latest completed reason: Watchdog, Image (boot/validation failure), None. History survives watchdog streak clearing and normal reboot.</t>
         </is>
       </c>
     </row>
@@ -32062,7 +32062,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Matching MCUboot/partition layout/signing key installed; current image Health=OK/60s; registered modem/data; configured HTTPS base URL; sufficient modem filesystem space. One update at a time.</t>
+          <t xml:space="preserve">Matching MCUboot/partition layout/signing key installed; startup health check disabled (Health=Off), no health wait; registered modem/data; configured HTTPS base URL; sufficient modem filesystem space. One update at a time.</t>
         </is>
       </c>
     </row>
@@ -32218,7 +32218,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Install the new project-key build-ota/merged.hex once via SWD, wait Health=OK/60s and Backup=Ready, then increment VERSION, build/sign using either project key and publish the DFU pair. Old SDK-signed 1.0.0/1.0.1 artifacts are not compatible with the new trust anchors.</t>
+          <t>Install the new project-key build-ota/merged.hex once via SWD, confirm Health=Off (no startup health wait), then increment VERSION, build/sign using either project key and publish the DFU pair. Old SDK-signed 1.0.0/1.0.1 artifacts are not compatible with the new trust anchors.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
improvements regarding speed of otas
</commit_message>
<xml_diff>
--- a/docs/SPS SMS Commands.xlsx
+++ b/docs/SPS SMS Commands.xlsx
@@ -31987,7 +31987,7 @@
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -32291,6 +32291,18 @@
       <c r="B25" t="inlineStr">
         <is>
           <t>Every MCU startup checks native HTTP state once after AT readiness/configuration. A stale or unknown HTTP state schedules cancellation/recovery without an OTA command; an idle modem is not reset. Normal modem polling and SMS submission wait until recovery completes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Storage phase and timing</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Saving firmware includes creating/reusing backup B, erasing staging A, modem-to-flash transfer and verification. Aligned image erases now use up to 64 KiB requests. Copy uses 1 KiB frames in batches up to 32 frames, checking a three-second budget between frames. OTA timing logs separate backup, staging erase, modem reads, flash writes, other copy work and verification. SMS times include cellular delays; speed improvements apply once the optimized updater is running.</t>
         </is>
       </c>
     </row>

</xml_diff>